<commit_message>
minor graph changes, also analysis done with new code
</commit_message>
<xml_diff>
--- a/NURBS IDX30 PYTHON ANALYSIS/Back_final_15_2_26/15gps/1mps_analysis.xlsx
+++ b/NURBS IDX30 PYTHON ANALYSIS/Back_final_15_2_26/15gps/1mps_analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Time</t>
   </si>
@@ -79,13 +79,34 @@
     <t>Q</t>
   </si>
   <si>
-    <t>rolling_std</t>
-  </si>
-  <si>
     <t>steady_state</t>
   </si>
   <si>
-    <t>avg_Q_steady</t>
+    <t>Averages</t>
+  </si>
+  <si>
+    <t>RTD_OUT_unc</t>
+  </si>
+  <si>
+    <t>RTD_IN_unc</t>
+  </si>
+  <si>
+    <t>RTD_unc</t>
+  </si>
+  <si>
+    <t>Delta_RTD</t>
+  </si>
+  <si>
+    <t>Rel_unc</t>
+  </si>
+  <si>
+    <t>ABS_unc</t>
+  </si>
+  <si>
+    <t>Average Q (W)</t>
+  </si>
+  <si>
+    <t>Average Q Uncertainty (W)</t>
   </si>
 </sst>
 </file>
@@ -421,10 +442,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X35"/>
+  <dimension ref="A1:AC35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:29">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -497,8 +518,23 @@
       <c r="X1" t="s">
         <v>23</v>
       </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:29">
       <c r="A2" s="1">
         <v>46068.53508956019</v>
       </c>
@@ -562,14 +598,32 @@
       <c r="U2">
         <v>214.6816001878013</v>
       </c>
-      <c r="W2" t="b">
+      <c r="V2" t="b">
         <v>0</v>
       </c>
+      <c r="W2" t="s">
+        <v>29</v>
+      </c>
       <c r="X2">
-        <v>217.3711893795659</v>
+        <v>0.254865552</v>
+      </c>
+      <c r="Y2">
+        <v>0.261409296</v>
+      </c>
+      <c r="Z2">
+        <v>0.3650907690307718</v>
+      </c>
+      <c r="AA2">
+        <v>3.271872000000002</v>
+      </c>
+      <c r="AB2">
+        <v>0.112031867663505</v>
+      </c>
+      <c r="AC2">
+        <v>24.05118062202925</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:29">
       <c r="A3" s="1">
         <v>46068.53520587963</v>
       </c>
@@ -633,11 +687,32 @@
       <c r="U3">
         <v>215.1051578837102</v>
       </c>
-      <c r="W3" t="b">
+      <c r="V3" t="b">
         <v>0</v>
       </c>
+      <c r="W3">
+        <v>217.5197871817224</v>
+      </c>
+      <c r="X3">
+        <v>0.254844246</v>
+      </c>
+      <c r="Y3">
+        <v>0.261403566</v>
+      </c>
+      <c r="Z3">
+        <v>0.3650717929898513</v>
+      </c>
+      <c r="AA3">
+        <v>3.27966</v>
+      </c>
+      <c r="AB3">
+        <v>0.1117621920518176</v>
+      </c>
+      <c r="AC3">
+        <v>24.04062396673577</v>
+      </c>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:29">
       <c r="A4" s="1">
         <v>46068.53532162037</v>
       </c>
@@ -701,14 +776,32 @@
       <c r="U4">
         <v>216.1208132384429</v>
       </c>
-      <c r="V4">
-        <v>0.7396272852477823</v>
-      </c>
-      <c r="W4" t="b">
-        <v>1</v>
+      <c r="V4" t="b">
+        <v>0</v>
+      </c>
+      <c r="W4" t="s">
+        <v>30</v>
+      </c>
+      <c r="X4">
+        <v>0.254810538</v>
+      </c>
+      <c r="Y4">
+        <v>0.26138797</v>
+      </c>
+      <c r="Z4">
+        <v>0.3650370955623145</v>
+      </c>
+      <c r="AA4">
+        <v>3.288716000000001</v>
+      </c>
+      <c r="AB4">
+        <v>0.1114463965033594</v>
+      </c>
+      <c r="AC4">
+        <v>24.0858858448</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:29">
       <c r="A5" s="1">
         <v>46068.53543793981</v>
       </c>
@@ -772,14 +865,32 @@
       <c r="U5">
         <v>216.3216937238412</v>
       </c>
-      <c r="V5">
-        <v>0.6521590065996559</v>
-      </c>
-      <c r="W5" t="b">
+      <c r="V5" t="b">
         <v>1</v>
       </c>
+      <c r="W5">
+        <v>24.09943133237424</v>
+      </c>
+      <c r="X5">
+        <v>0.254823576</v>
+      </c>
+      <c r="Y5">
+        <v>0.261396882</v>
+      </c>
+      <c r="Z5">
+        <v>0.3650525781373824</v>
+      </c>
+      <c r="AA5">
+        <v>3.286653000000001</v>
+      </c>
+      <c r="AB5">
+        <v>0.1115204790364601</v>
+      </c>
+      <c r="AC5">
+        <v>24.12429891006117</v>
+      </c>
     </row>
-    <row r="6" spans="1:24">
+    <row r="6" spans="1:29">
       <c r="A6" s="1">
         <v>46068.53555368056</v>
       </c>
@@ -843,14 +954,29 @@
       <c r="U6">
         <v>216.728507456018</v>
       </c>
-      <c r="V6">
-        <v>0.3096079898236418</v>
-      </c>
-      <c r="W6" t="b">
+      <c r="V6" t="b">
         <v>1</v>
       </c>
+      <c r="X6">
+        <v>0.25479464</v>
+      </c>
+      <c r="Y6">
+        <v>0.26139561</v>
+      </c>
+      <c r="Z6">
+        <v>0.3650314691913585</v>
+      </c>
+      <c r="AA6">
+        <v>3.300485000000002</v>
+      </c>
+      <c r="AB6">
+        <v>0.1110505040278246</v>
+      </c>
+      <c r="AC6">
+        <v>24.06780999018894</v>
+      </c>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:29">
       <c r="A7" s="1">
         <v>46068.53567</v>
       </c>
@@ -914,14 +1040,29 @@
       <c r="U7">
         <v>217.2155233861974</v>
       </c>
-      <c r="V7">
-        <v>0.447514132783167</v>
-      </c>
-      <c r="W7" t="b">
+      <c r="V7" t="b">
         <v>1</v>
       </c>
+      <c r="X7">
+        <v>0.25478828</v>
+      </c>
+      <c r="Y7">
+        <v>0.261398792</v>
+      </c>
+      <c r="Z7">
+        <v>0.3650293085279833</v>
+      </c>
+      <c r="AA7">
+        <v>3.305256</v>
+      </c>
+      <c r="AB7">
+        <v>0.1108908569410966</v>
+      </c>
+      <c r="AC7">
+        <v>24.08721552920424</v>
+      </c>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:29">
       <c r="A8" s="1">
         <v>46068.53578631944</v>
       </c>
@@ -985,14 +1126,29 @@
       <c r="U8">
         <v>218.0938148388553</v>
       </c>
-      <c r="V8">
-        <v>0.6919350453246611</v>
-      </c>
-      <c r="W8" t="b">
+      <c r="V8" t="b">
         <v>1</v>
       </c>
+      <c r="X8">
+        <v>0.254784782</v>
+      </c>
+      <c r="Y8">
+        <v>0.261394018</v>
+      </c>
+      <c r="Z8">
+        <v>0.3650234482673296</v>
+      </c>
+      <c r="AA8">
+        <v>3.304617999999998</v>
+      </c>
+      <c r="AB8">
+        <v>0.1109103256630352</v>
+      </c>
+      <c r="AC8">
+        <v>24.18885602887114</v>
+      </c>
     </row>
-    <row r="9" spans="1:24">
+    <row r="9" spans="1:29">
       <c r="A9" s="1">
         <v>46068.53590206018</v>
       </c>
@@ -1056,14 +1212,29 @@
       <c r="U9">
         <v>217.9789494872676</v>
       </c>
-      <c r="V9">
-        <v>0.4773903602928023</v>
-      </c>
-      <c r="W9" t="b">
+      <c r="V9" t="b">
         <v>1</v>
       </c>
+      <c r="X9">
+        <v>0.2547851</v>
+      </c>
+      <c r="Y9">
+        <v>0.261398792</v>
+      </c>
+      <c r="Z9">
+        <v>0.3650270889140548</v>
+      </c>
+      <c r="AA9">
+        <v>3.306846</v>
+      </c>
+      <c r="AB9">
+        <v>0.1108373035431468</v>
+      </c>
+      <c r="AC9">
+        <v>24.16019899033655</v>
+      </c>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:29">
       <c r="A10" s="1">
         <v>46068.53601780093</v>
       </c>
@@ -1127,14 +1298,29 @@
       <c r="U10">
         <v>217.3344766572664</v>
       </c>
-      <c r="V10">
-        <v>0.4092948716235621</v>
-      </c>
-      <c r="W10" t="b">
+      <c r="V10" t="b">
         <v>1</v>
       </c>
+      <c r="X10">
+        <v>0.254775878</v>
+      </c>
+      <c r="Y10">
+        <v>0.261399428</v>
+      </c>
+      <c r="Z10">
+        <v>0.3650211075669434</v>
+      </c>
+      <c r="AA10">
+        <v>3.311774999999997</v>
+      </c>
+      <c r="AB10">
+        <v>0.1106718866281937</v>
+      </c>
+      <c r="AC10">
+        <v>24.0528165610108</v>
+      </c>
     </row>
-    <row r="11" spans="1:24">
+    <row r="11" spans="1:29">
       <c r="A11" s="1">
         <v>46068.53613412037</v>
       </c>
@@ -1198,14 +1384,29 @@
       <c r="U11">
         <v>218.4579458959465</v>
       </c>
-      <c r="V11">
-        <v>0.5637620535884865</v>
-      </c>
-      <c r="W11" t="b">
+      <c r="V11" t="b">
         <v>1</v>
       </c>
+      <c r="X11">
+        <v>0.254773652</v>
+      </c>
+      <c r="Y11">
+        <v>0.261405794</v>
+      </c>
+      <c r="Z11">
+        <v>0.3650241127517297</v>
+      </c>
+      <c r="AA11">
+        <v>3.316071000000001</v>
+      </c>
+      <c r="AB11">
+        <v>0.1105305840677204</v>
+      </c>
+      <c r="AC11">
+        <v>24.14628435411344</v>
+      </c>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:29">
       <c r="A12" s="1">
         <v>46068.53625043981</v>
       </c>
@@ -1269,14 +1470,29 @@
       <c r="U12">
         <v>218.4772319178293</v>
       </c>
-      <c r="V12">
-        <v>0.6542737279413</v>
-      </c>
-      <c r="W12" t="b">
+      <c r="V12" t="b">
         <v>1</v>
       </c>
+      <c r="X12">
+        <v>0.254758388</v>
+      </c>
+      <c r="Y12">
+        <v>0.261400702</v>
+      </c>
+      <c r="Z12">
+        <v>0.3650098125563905</v>
+      </c>
+      <c r="AA12">
+        <v>3.321156999999999</v>
+      </c>
+      <c r="AB12">
+        <v>0.110358416664149</v>
+      </c>
+      <c r="AC12">
+        <v>24.11080139161772</v>
+      </c>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:29">
       <c r="A13" s="1">
         <v>46068.53636618055</v>
       </c>
@@ -1340,14 +1556,29 @@
       <c r="U13">
         <v>217.577231012925</v>
       </c>
-      <c r="V13">
-        <v>0.5141388082098938</v>
-      </c>
-      <c r="W13" t="b">
+      <c r="V13" t="b">
         <v>1</v>
       </c>
+      <c r="X13">
+        <v>0.254771108</v>
+      </c>
+      <c r="Y13">
+        <v>0.261392108</v>
+      </c>
+      <c r="Z13">
+        <v>0.3650125362179104</v>
+      </c>
+      <c r="AA13">
+        <v>3.310499999999998</v>
+      </c>
+      <c r="AB13">
+        <v>0.1107115841083422</v>
+      </c>
+      <c r="AC13">
+        <v>24.08831991134765</v>
+      </c>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:29">
       <c r="A14" s="1">
         <v>46068.5364819213</v>
       </c>
@@ -1411,14 +1642,29 @@
       <c r="U14">
         <v>217.1565102373447</v>
       </c>
-      <c r="V14">
-        <v>0.6746991128317513</v>
-      </c>
-      <c r="W14" t="b">
+      <c r="V14" t="b">
         <v>1</v>
       </c>
+      <c r="X14">
+        <v>0.254770472</v>
+      </c>
+      <c r="Y14">
+        <v>0.261382878</v>
+      </c>
+      <c r="Z14">
+        <v>0.3650054825816534</v>
+      </c>
+      <c r="AA14">
+        <v>3.306203000000004</v>
+      </c>
+      <c r="AB14">
+        <v>0.1108521756092177</v>
+      </c>
+      <c r="AC14">
+        <v>24.07227160751501</v>
+      </c>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:29">
       <c r="A15" s="1">
         <v>46068.53659824074</v>
       </c>
@@ -1482,14 +1728,29 @@
       <c r="U15">
         <v>218.1237053581147</v>
       </c>
-      <c r="V15">
-        <v>0.4849581739003441</v>
-      </c>
-      <c r="W15" t="b">
+      <c r="V15" t="b">
         <v>1</v>
       </c>
+      <c r="X15">
+        <v>0.254752028</v>
+      </c>
+      <c r="Y15">
+        <v>0.261388288</v>
+      </c>
+      <c r="Z15">
+        <v>0.3649964833716672</v>
+      </c>
+      <c r="AA15">
+        <v>3.318130000000004</v>
+      </c>
+      <c r="AB15">
+        <v>0.1104542654822624</v>
+      </c>
+      <c r="AC15">
+        <v>24.09269365959997</v>
+      </c>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:29">
       <c r="A16" s="1">
         <v>46068.53671398148</v>
       </c>
@@ -1553,14 +1814,29 @@
       <c r="U16">
         <v>217.9331409181729</v>
       </c>
-      <c r="V16">
-        <v>0.5123371972011092</v>
-      </c>
-      <c r="W16" t="b">
+      <c r="V16" t="b">
         <v>1</v>
       </c>
+      <c r="X16">
+        <v>0.254764748</v>
+      </c>
+      <c r="Y16">
+        <v>0.261388606</v>
+      </c>
+      <c r="Z16">
+        <v>0.3650055892313524</v>
+      </c>
+      <c r="AA16">
+        <v>3.311928999999999</v>
+      </c>
+      <c r="AB16">
+        <v>0.1106621161393435</v>
+      </c>
+      <c r="AC16">
+        <v>24.11694255089876</v>
+      </c>
     </row>
-    <row r="17" spans="1:23">
+    <row r="17" spans="1:29">
       <c r="A17" s="1">
         <v>46068.53683030092</v>
       </c>
@@ -1624,14 +1900,29 @@
       <c r="U17">
         <v>217.5646314057498</v>
       </c>
-      <c r="V17">
-        <v>0.284217566525393</v>
-      </c>
-      <c r="W17" t="b">
+      <c r="V17" t="b">
         <v>1</v>
       </c>
+      <c r="X17">
+        <v>0.254753618</v>
+      </c>
+      <c r="Y17">
+        <v>0.261381286</v>
+      </c>
+      <c r="Z17">
+        <v>0.3649925787671631</v>
+      </c>
+      <c r="AA17">
+        <v>3.313834</v>
+      </c>
+      <c r="AB17">
+        <v>0.1105951102013323</v>
+      </c>
+      <c r="AC17">
+        <v>24.06158438623113</v>
+      </c>
     </row>
-    <row r="18" spans="1:23">
+    <row r="18" spans="1:29">
       <c r="A18" s="1">
         <v>46068.53694604167</v>
       </c>
@@ -1695,14 +1986,29 @@
       <c r="U18">
         <v>218.8398208852459</v>
       </c>
-      <c r="V18">
-        <v>0.6562489405776417</v>
-      </c>
-      <c r="W18" t="b">
+      <c r="V18" t="b">
         <v>1</v>
       </c>
+      <c r="X18">
+        <v>0.25475966</v>
+      </c>
+      <c r="Y18">
+        <v>0.261400384</v>
+      </c>
+      <c r="Z18">
+        <v>0.3650104726150512</v>
+      </c>
+      <c r="AA18">
+        <v>3.320362000000003</v>
+      </c>
+      <c r="AB18">
+        <v>0.110384821011407</v>
+      </c>
+      <c r="AC18">
+        <v>24.15659445858624</v>
+      </c>
     </row>
-    <row r="19" spans="1:23">
+    <row r="19" spans="1:29">
       <c r="A19" s="1">
         <v>46068.53706236111</v>
       </c>
@@ -1766,14 +2072,29 @@
       <c r="U19">
         <v>218.1466144032881</v>
       </c>
-      <c r="V19">
-        <v>0.63840264784721</v>
-      </c>
-      <c r="W19" t="b">
+      <c r="V19" t="b">
         <v>1</v>
       </c>
+      <c r="X19">
+        <v>0.254750756</v>
+      </c>
+      <c r="Y19">
+        <v>0.26138988</v>
+      </c>
+      <c r="Z19">
+        <v>0.3649967356689453</v>
+      </c>
+      <c r="AA19">
+        <v>3.319562000000005</v>
+      </c>
+      <c r="AB19">
+        <v>0.1104070838040025</v>
+      </c>
+      <c r="AC19">
+        <v>24.08493153798326</v>
+      </c>
     </row>
-    <row r="20" spans="1:23">
+    <row r="20" spans="1:29">
       <c r="A20" s="1">
         <v>46068.53717868056</v>
       </c>
@@ -1837,14 +2158,29 @@
       <c r="U20">
         <v>218.0263851157382</v>
       </c>
-      <c r="V20">
-        <v>0.4390649267341463</v>
-      </c>
-      <c r="W20" t="b">
+      <c r="V20" t="b">
         <v>1</v>
       </c>
+      <c r="X20">
+        <v>0.254747578</v>
+      </c>
+      <c r="Y20">
+        <v>0.261368236</v>
+      </c>
+      <c r="Z20">
+        <v>0.3649790175977488</v>
+      </c>
+      <c r="AA20">
+        <v>3.310328999999996</v>
+      </c>
+      <c r="AB20">
+        <v>0.1107071723473693</v>
+      </c>
+      <c r="AC20">
+        <v>24.13708459328194</v>
+      </c>
     </row>
-    <row r="21" spans="1:23">
+    <row r="21" spans="1:29">
       <c r="A21" s="1">
         <v>46068.537295</v>
       </c>
@@ -1908,14 +2244,29 @@
       <c r="U21">
         <v>218.1750744293984</v>
       </c>
-      <c r="V21">
-        <v>0.07892355654707837</v>
-      </c>
-      <c r="W21" t="b">
+      <c r="V21" t="b">
         <v>1</v>
       </c>
+      <c r="X21">
+        <v>0.254742808</v>
+      </c>
+      <c r="Y21">
+        <v>0.261379058</v>
+      </c>
+      <c r="Z21">
+        <v>0.3649834382389045</v>
+      </c>
+      <c r="AA21">
+        <v>3.318125000000002</v>
+      </c>
+      <c r="AB21">
+        <v>0.1104505152277</v>
+      </c>
+      <c r="AC21">
+        <v>24.09754938056884</v>
+      </c>
     </row>
-    <row r="22" spans="1:23">
+    <row r="22" spans="1:29">
       <c r="A22" s="1">
         <v>46068.53741074074</v>
       </c>
@@ -1979,14 +2330,29 @@
       <c r="U22">
         <v>217.6430559034833</v>
       </c>
-      <c r="V22">
-        <v>0.2744975740274997</v>
-      </c>
-      <c r="W22" t="b">
+      <c r="V22" t="b">
         <v>1</v>
       </c>
+      <c r="X22">
+        <v>0.2547692</v>
+      </c>
+      <c r="Y22">
+        <v>0.261376194</v>
+      </c>
+      <c r="Z22">
+        <v>0.3649998082993547</v>
+      </c>
+      <c r="AA22">
+        <v>3.303497</v>
+      </c>
+      <c r="AB22">
+        <v>0.1109405288619105</v>
+      </c>
+      <c r="AC22">
+        <v>24.14543572505478</v>
+      </c>
     </row>
-    <row r="23" spans="1:23">
+    <row r="23" spans="1:29">
       <c r="A23" s="1">
         <v>46068.53752648148</v>
       </c>
@@ -2050,14 +2416,29 @@
       <c r="U23">
         <v>217.5430496176586</v>
       </c>
-      <c r="V23">
-        <v>0.3397303665595646</v>
-      </c>
-      <c r="W23" t="b">
+      <c r="V23" t="b">
         <v>1</v>
       </c>
+      <c r="X23">
+        <v>0.254770472</v>
+      </c>
+      <c r="Y23">
+        <v>0.261387652</v>
+      </c>
+      <c r="Z23">
+        <v>0.3650089012903328</v>
+      </c>
+      <c r="AA23">
+        <v>3.308590000000002</v>
+      </c>
+      <c r="AB23">
+        <v>0.110773880835855</v>
+      </c>
+      <c r="AC23">
+        <v>24.098087855015</v>
+      </c>
     </row>
-    <row r="24" spans="1:23">
+    <row r="24" spans="1:29">
       <c r="A24" s="1">
         <v>46068.53764222223</v>
       </c>
@@ -2121,14 +2502,29 @@
       <c r="U24">
         <v>218.14620668762</v>
       </c>
-      <c r="V24">
-        <v>0.3232543940991266</v>
-      </c>
-      <c r="W24" t="b">
+      <c r="V24" t="b">
         <v>1</v>
       </c>
+      <c r="X24">
+        <v>0.254769518</v>
+      </c>
+      <c r="Y24">
+        <v>0.261396882</v>
+      </c>
+      <c r="Z24">
+        <v>0.3650148452067042</v>
+      </c>
+      <c r="AA24">
+        <v>3.313682</v>
+      </c>
+      <c r="AB24">
+        <v>0.1106068337963102</v>
+      </c>
+      <c r="AC24">
+        <v>24.12846122639312</v>
+      </c>
     </row>
-    <row r="25" spans="1:23">
+    <row r="25" spans="1:29">
       <c r="A25" s="1">
         <v>46068.53775854166</v>
       </c>
@@ -2192,14 +2588,29 @@
       <c r="U25">
         <v>217.4917034097112</v>
       </c>
-      <c r="V25">
-        <v>0.3639618626789619</v>
-      </c>
-      <c r="W25" t="b">
+      <c r="V25" t="b">
         <v>1</v>
       </c>
+      <c r="X25">
+        <v>0.254785418</v>
+      </c>
+      <c r="Y25">
+        <v>0.261402612</v>
+      </c>
+      <c r="Z25">
+        <v>0.3650300464151647</v>
+      </c>
+      <c r="AA25">
+        <v>3.308596999999999</v>
+      </c>
+      <c r="AB25">
+        <v>0.1107800132524768</v>
+      </c>
+      <c r="AC25">
+        <v>24.09373378603156</v>
+      </c>
     </row>
-    <row r="26" spans="1:23">
+    <row r="26" spans="1:29">
       <c r="A26" s="1">
         <v>46068.53787486111</v>
       </c>
@@ -2263,14 +2674,29 @@
       <c r="U26">
         <v>217.6027482215071</v>
       </c>
-      <c r="V26">
-        <v>0.3502505282913006</v>
-      </c>
-      <c r="W26" t="b">
+      <c r="V26" t="b">
         <v>1</v>
       </c>
+      <c r="X26">
+        <v>0.25477397</v>
+      </c>
+      <c r="Y26">
+        <v>0.261402294</v>
+      </c>
+      <c r="Z26">
+        <v>0.3650218282486998</v>
+      </c>
+      <c r="AA26">
+        <v>3.314161999999996</v>
+      </c>
+      <c r="AB26">
+        <v>0.1105930436304938</v>
+      </c>
+      <c r="AC26">
+        <v>24.06535022817649</v>
+      </c>
     </row>
-    <row r="27" spans="1:23">
+    <row r="27" spans="1:29">
       <c r="A27" s="1">
         <v>46068.53799060185</v>
       </c>
@@ -2334,14 +2760,29 @@
       <c r="U27">
         <v>217.3178595498872</v>
       </c>
-      <c r="V27">
-        <v>0.1435932873561181</v>
-      </c>
-      <c r="W27" t="b">
+      <c r="V27" t="b">
         <v>1</v>
       </c>
+      <c r="X27">
+        <v>0.25479782</v>
+      </c>
+      <c r="Y27">
+        <v>0.261420754</v>
+      </c>
+      <c r="Z27">
+        <v>0.3650516945566489</v>
+      </c>
+      <c r="AA27">
+        <v>3.311467</v>
+      </c>
+      <c r="AB27">
+        <v>0.1106912951135006</v>
+      </c>
+      <c r="AC27">
+        <v>24.05519532487083</v>
+      </c>
     </row>
-    <row r="28" spans="1:23">
+    <row r="28" spans="1:29">
       <c r="A28" s="1">
         <v>46068.5381063426</v>
       </c>
@@ -2405,14 +2846,29 @@
       <c r="U28">
         <v>217.6452366858863</v>
       </c>
-      <c r="V28">
-        <v>0.1780180767962433</v>
-      </c>
-      <c r="W28" t="b">
+      <c r="V28" t="b">
         <v>1</v>
       </c>
+      <c r="X28">
+        <v>0.254806722</v>
+      </c>
+      <c r="Y28">
+        <v>0.26142712</v>
+      </c>
+      <c r="Z28">
+        <v>0.3650624667750434</v>
+      </c>
+      <c r="AA28">
+        <v>3.310199000000004</v>
+      </c>
+      <c r="AB28">
+        <v>0.1107365913194495</v>
+      </c>
+      <c r="AC28">
+        <v>24.10129162750984</v>
+      </c>
     </row>
-    <row r="29" spans="1:23">
+    <row r="29" spans="1:29">
       <c r="A29" s="1">
         <v>46068.53822266203</v>
       </c>
@@ -2476,14 +2932,29 @@
       <c r="U29">
         <v>217.0010598297539</v>
       </c>
-      <c r="V29">
-        <v>0.3221029012152638</v>
-      </c>
-      <c r="W29" t="b">
+      <c r="V29" t="b">
         <v>1</v>
       </c>
+      <c r="X29">
+        <v>0.25483407</v>
+      </c>
+      <c r="Y29">
+        <v>0.261433804</v>
+      </c>
+      <c r="Z29">
+        <v>0.3650863419886798</v>
+      </c>
+      <c r="AA29">
+        <v>3.299866999999999</v>
+      </c>
+      <c r="AB29">
+        <v>0.1110876942366666</v>
+      </c>
+      <c r="AC29">
+        <v>24.1061473834003</v>
+      </c>
     </row>
-    <row r="30" spans="1:23">
+    <row r="30" spans="1:29">
       <c r="A30" s="1">
         <v>46068.53833898148</v>
       </c>
@@ -2547,14 +3018,29 @@
       <c r="U30">
         <v>216.8056177904474</v>
       </c>
-      <c r="V30">
-        <v>0.4393406617273984</v>
-      </c>
-      <c r="W30" t="b">
+      <c r="V30" t="b">
         <v>1</v>
       </c>
+      <c r="X30">
+        <v>0.254836614</v>
+      </c>
+      <c r="Y30">
+        <v>0.261444306</v>
+      </c>
+      <c r="Z30">
+        <v>0.3650956381207623</v>
+      </c>
+      <c r="AA30">
+        <v>3.303846</v>
+      </c>
+      <c r="AB30">
+        <v>0.1109577924077688</v>
+      </c>
+      <c r="AC30">
+        <v>24.05627273163052</v>
+      </c>
     </row>
-    <row r="31" spans="1:23">
+    <row r="31" spans="1:29">
       <c r="A31" s="1">
         <v>46068.53845530093</v>
       </c>
@@ -2618,14 +3104,29 @@
       <c r="U31">
         <v>217.180363365064</v>
       </c>
-      <c r="V31">
-        <v>0.1874306957238331</v>
-      </c>
-      <c r="W31" t="b">
+      <c r="V31" t="b">
         <v>1</v>
       </c>
+      <c r="X31">
+        <v>0.254824212</v>
+      </c>
+      <c r="Y31">
+        <v>0.261445262</v>
+      </c>
+      <c r="Z31">
+        <v>0.3650876662442455</v>
+      </c>
+      <c r="AA31">
+        <v>3.310524999999998</v>
+      </c>
+      <c r="AB31">
+        <v>0.1107333564169285</v>
+      </c>
+      <c r="AC31">
+        <v>24.04911058326167</v>
+      </c>
     </row>
-    <row r="32" spans="1:23">
+    <row r="32" spans="1:29">
       <c r="A32" s="1">
         <v>46068.53857162037</v>
       </c>
@@ -2689,14 +3190,29 @@
       <c r="U32">
         <v>217.5498003565519</v>
       </c>
-      <c r="V32">
-        <v>0.3720944387445765</v>
-      </c>
-      <c r="W32" t="b">
+      <c r="V32" t="b">
         <v>1</v>
       </c>
+      <c r="X32">
+        <v>0.25483566</v>
+      </c>
+      <c r="Y32">
+        <v>0.261448762</v>
+      </c>
+      <c r="Z32">
+        <v>0.3650981631821342</v>
+      </c>
+      <c r="AA32">
+        <v>3.306550999999999</v>
+      </c>
+      <c r="AB32">
+        <v>0.1108685189607152</v>
+      </c>
+      <c r="AC32">
+        <v>24.11942416573018</v>
+      </c>
     </row>
-    <row r="33" spans="1:23">
+    <row r="33" spans="1:29">
       <c r="A33" s="1">
         <v>46068.53868736111</v>
       </c>
@@ -2760,14 +3276,29 @@
       <c r="U33">
         <v>216.5307421123249</v>
       </c>
-      <c r="V33">
-        <v>0.5159087722676492</v>
-      </c>
-      <c r="W33" t="b">
+      <c r="V33" t="b">
         <v>1</v>
       </c>
+      <c r="X33">
+        <v>0.25485951</v>
+      </c>
+      <c r="Y33">
+        <v>0.26145672</v>
+      </c>
+      <c r="Z33">
+        <v>0.3651205092440008</v>
+      </c>
+      <c r="AA33">
+        <v>3.298605000000002</v>
+      </c>
+      <c r="AB33">
+        <v>0.1111401665704277</v>
+      </c>
+      <c r="AC33">
+        <v>24.06526274598211</v>
+      </c>
     </row>
-    <row r="34" spans="1:23">
+    <row r="34" spans="1:29">
       <c r="A34" s="1">
         <v>46068.53880310185</v>
       </c>
@@ -2831,14 +3362,29 @@
       <c r="U34">
         <v>215.7944970286389</v>
       </c>
-      <c r="V34">
-        <v>0.8814407052622998</v>
-      </c>
-      <c r="W34" t="b">
+      <c r="V34" t="b">
         <v>1</v>
       </c>
+      <c r="X34">
+        <v>0.254879224</v>
+      </c>
+      <c r="Y34">
+        <v>0.26146786</v>
+      </c>
+      <c r="Z34">
+        <v>0.3651422471309253</v>
+      </c>
+      <c r="AA34">
+        <v>3.294318000000004</v>
+      </c>
+      <c r="AB34">
+        <v>0.1112901985459643</v>
+      </c>
+      <c r="AC34">
+        <v>24.01581241944373</v>
+      </c>
     </row>
-    <row r="35" spans="1:23">
+    <row r="35" spans="1:29">
       <c r="A35" s="1">
         <v>46068.5389194213</v>
       </c>
@@ -2902,11 +3448,26 @@
       <c r="U35">
         <v>216.7102049456601</v>
       </c>
-      <c r="V35">
-        <v>0.4852464530342937</v>
-      </c>
-      <c r="W35" t="b">
+      <c r="V35" t="b">
         <v>1</v>
+      </c>
+      <c r="X35">
+        <v>0.254885266</v>
+      </c>
+      <c r="Y35">
+        <v>0.261468814</v>
+      </c>
+      <c r="Z35">
+        <v>0.3651471477616351</v>
+      </c>
+      <c r="AA35">
+        <v>3.291773999999997</v>
+      </c>
+      <c r="AB35">
+        <v>0.1113769961397835</v>
+      </c>
+      <c r="AC35">
+        <v>24.13653165968447</v>
       </c>
     </row>
   </sheetData>

</xml_diff>